<commit_message>
ПМИ tkzdz и torpn
</commit_message>
<xml_diff>
--- a/PMI-DZT2/ПМИ ТокЗ/pmi_tokzdzt/tkzdz_mode/ТК ЗДЗ_1.xlsx
+++ b/PMI-DZT2/ПМИ ТокЗ/pmi_tokzdzt/tkzdz_mode/ТК ЗДЗ_1.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,18 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -46,7 +58,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -60,16 +72,37 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,97 +472,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_hvptoc1_strtpalc</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc1_strtpalc</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc2_strtpalc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_palc1_eqpalc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>SGF2_palc1_eqpalc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>SGF3_palc1_eqpalc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_EnaDis</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>LVARCTOC_1_PTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>LTCBLKTOC_1_PTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_HVPTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC2_EnaDis</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>TPALC_1_HVPTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC2_EnaDis</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_CurrCtrlEna</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_OilTmpCtrlEna</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_PTRC1_EnaDis</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_RBRE1_EnaDis</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Номинальный ток входа ВН</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Номинальный ток входа НН1</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Номинальный ток входа НН2</t>
         </is>
@@ -609,79 +642,79 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>T1_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>T1_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>T1_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_hvptoc1_strtpalc</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc1_strtpalc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc2_strtpalc</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>T1_palc1_eqpalc</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_Top</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_Top</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_Top</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_Iop</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>LVARCTOC_1_PTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>LTCBLKTOC_1_PTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_HVPTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC2_Iop</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_HVPTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC1_Iop</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC2_Iop</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_Top</t>
         </is>
       </c>
     </row>
@@ -778,149 +811,149 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>IB</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>IA1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>IB1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>IC1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>VYVOD</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>OV_tovctoc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>OV_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>NaOtkl_tovctoc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>OV_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>OV_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>OV_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>OV_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>OV_strpalc</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>OV_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>OV_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>OV_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>OV_tpalc</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>OV_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>OV_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>OV_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>OV_eqpalc</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>NaSign_eqpalc</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>otkaz_so</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>t_masla_zpo</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>OV_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>OV_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>OV_rbre1_tprmofflvlgc</t>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>DI_ControllerDisable</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TOVCTOC</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TOVCTOC_HVPTOC1</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>DI_TOVCTOC_Sign</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TOVCTOC_LVPTOC1</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TOVCTOC_LVPTOC2</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>DI_LVARCTOC</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>DI_LTCBLKTOC</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>DI_STRTPALC</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>DI_STRTPALC_HVPTOC1</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>DI_STRTPALC_LVPTOC1</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>DI_STRTPALC_LVPTOC2</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TPALC</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TPALC_HVPTOC1</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TPALC_LVPTOC1</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TPALC_LVPTOC2</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>DI_EQPALC</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>DI_EQPALC_Sign</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>FailCoolSys</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>AlcOilTmp</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TPRMOFFLVLGC</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>DI_TJNTPTRC</t>
+        </is>
+      </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>DI_JNTRBRE</t>
         </is>
       </c>
     </row>
@@ -1098,344 +1131,344 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>io_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>srab_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>srabotkl_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>io_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>srab_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>srabotkl_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>io_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>srab_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>srabotkl_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>srab_tovctoc</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>io_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>io_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>io_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>io_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>io_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_strpalc</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_strpalc</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>io_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>io_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>io_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_tpalc</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_tpalc</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>srabsign_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>srab_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_Str</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_Op</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_HVPTOC1_OpOnTrip</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_Str</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_Op</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC1_OpOnTrip</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_Str</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_DE_I</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_Op</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_PTOC2_OpOnTrip</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>TOVCTOC_1_TOVCTOC_Op</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>LVARCTOC_1_PTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>LVARCTOC_1_PTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>LVARCTOC_1_PTOC1_Str</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>LVARCTOC_1_PTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>LTCBLKTOC_1_PTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>LTCBLKTOC_1_PTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>LTCBLKTOC_1_PTOC1_Str</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>LTCBLKTOC_1_PTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_HVPTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_HVPTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="AD1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_HVPTOC1_Str</t>
+        </is>
+      </c>
+      <c r="AE1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_HVPTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="AF1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AG1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="AH1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC1_Str</t>
+        </is>
+      </c>
+      <c r="AI1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="AJ1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC2_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AK1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC2_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="AL1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC2_Str</t>
+        </is>
+      </c>
+      <c r="AM1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_LVPTOC2_DE_I</t>
+        </is>
+      </c>
+      <c r="AN1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_PTOC1_Str</t>
+        </is>
+      </c>
+      <c r="AO1" s="4" t="inlineStr">
+        <is>
+          <t>STRTPALC_1_PTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AP1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_HVPTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AQ1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_HVPTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="AR1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_HVPTOC1_Str</t>
+        </is>
+      </c>
+      <c r="AS1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_HVPTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="AT1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AU1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="AV1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC1_Str</t>
+        </is>
+      </c>
+      <c r="AW1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC1_DE_I</t>
+        </is>
+      </c>
+      <c r="AX1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC2_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="AY1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC2_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="AZ1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC2_Str</t>
+        </is>
+      </c>
+      <c r="BA1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_LVPTOC2_DE_I</t>
+        </is>
+      </c>
+      <c r="BB1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_PTOC1_Str</t>
+        </is>
+      </c>
+      <c r="BC1" s="4" t="inlineStr">
+        <is>
+          <t>TPALC_1_PTOC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="BD1" s="4" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="BE1" s="4" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="BF1" s="4" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_Str</t>
+        </is>
+      </c>
+      <c r="BG1" s="4" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_OpOnSignal</t>
+        </is>
+      </c>
+      <c r="BH1" s="4" t="inlineStr">
+        <is>
+          <t>EQPALC_1_PALC1_Op</t>
+        </is>
+      </c>
+      <c r="BI1" s="4" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_PTRC1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="BJ1" s="4" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_PTRC1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="BK1" s="3" t="inlineStr">
         <is>
           <t>pusk_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>srab_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
-        <is>
-          <t>zapret_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BP1" s="1" t="inlineStr">
-        <is>
-          <t>pusk_lvalh</t>
+      <c r="BL1" s="4" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_PTRC1_Op</t>
+        </is>
+      </c>
+      <c r="BM1" s="4" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_RBRE1_FuncEnabled</t>
+        </is>
+      </c>
+      <c r="BN1" s="4" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_RBRE1_FuncOperDisabled</t>
+        </is>
+      </c>
+      <c r="BO1" s="4" t="inlineStr">
+        <is>
+          <t>TPRMOFFLVLGC_1_RBRE1_BlkOp</t>
+        </is>
+      </c>
+      <c r="BP1" s="4" t="inlineStr">
+        <is>
+          <t>DZT2_LVALH_1_CALH1_Alarm</t>
         </is>
       </c>
     </row>

</xml_diff>